<commit_message>
fixed show difference logic
</commit_message>
<xml_diff>
--- a/client-course-schedulizer/csv/test_mutiple/3_mutiple_in_one_row.xlsx
+++ b/client-course-schedulizer/csv/test_mutiple/3_mutiple_in_one_row.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\李约瑟\Desktop\sen\course-schedulizer\client-course-schedulizer\csv\test_mutiple\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B610570-745E-4EC0-B0E5-13E53535D8A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4031444C-18C7-4068-9D97-5A17E0861AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1368" yWindow="696" windowWidth="39912" windowHeight="16584" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="98">
   <si>
     <t>Department</t>
   </si>
@@ -181,6 +181,9 @@
     <t>13:30:00</t>
   </si>
   <si>
+    <t>E</t>
+  </si>
+  <si>
     <t>John Ferdinands</t>
   </si>
   <si>
@@ -307,19 +310,11 @@
     <t>NH 120</t>
   </si>
   <si>
-    <t>E</t>
+    <t>FA</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>yuyuyuyuyu</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>B</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>James Turner</t>
+    <t>YUESE LEYYYYY</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -904,13 +899,13 @@
         <v>26</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>98</v>
+        <v>81</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="I2" s="2">
         <v>4</v>
@@ -925,14 +920,14 @@
       <c r="M2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="N2" s="2">
-        <v>15</v>
+      <c r="N2" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>41</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>29</v>
@@ -976,7 +971,7 @@
         <v>27</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I3" s="2">
         <v>4</v>
@@ -1042,7 +1037,7 @@
         <v>32</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I4" s="2">
         <v>4</v>
@@ -1061,7 +1056,7 @@
         <v>38</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>45</v>
@@ -1102,7 +1097,7 @@
         <v>26</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>27</v>
@@ -1130,7 +1125,7 @@
         <v>48</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>29</v>
@@ -1168,7 +1163,7 @@
         <v>26</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>32</v>
@@ -1196,7 +1191,7 @@
         <v>48</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>29</v>
@@ -1234,7 +1229,7 @@
         <v>26</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>49</v>
@@ -1259,10 +1254,10 @@
         <v>38</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>29</v>
@@ -1300,13 +1295,13 @@
         <v>26</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I8" s="2">
         <v>4</v>
@@ -1325,16 +1320,16 @@
         <v>38</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>29</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="S8" s="2" t="s">
         <v>31</v>
@@ -1366,7 +1361,7 @@
         <v>26</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>27</v>
@@ -1391,16 +1386,16 @@
         <v>38</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>29</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="S9" s="2" t="s">
         <v>31</v>
@@ -1432,7 +1427,7 @@
         <v>26</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>27</v>
@@ -1460,13 +1455,13 @@
         <v>41</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q10" s="2" t="s">
         <v>29</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="S10" s="2" t="s">
         <v>31</v>
@@ -1498,7 +1493,7 @@
         <v>26</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>32</v>
@@ -1526,13 +1521,13 @@
         <v>41</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>29</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="S11" s="2" t="s">
         <v>31</v>
@@ -1564,13 +1559,13 @@
         <v>26</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>49</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I12" s="2">
         <v>4</v>
@@ -1592,13 +1587,13 @@
         <v>35</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>29</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="S12" s="2" t="s">
         <v>31</v>
@@ -1630,13 +1625,13 @@
         <v>26</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I13" s="2">
         <v>4</v>
@@ -1658,13 +1653,13 @@
         <v>41</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q13" s="2" t="s">
         <v>29</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="S13" s="2" t="s">
         <v>31</v>
@@ -1696,13 +1691,13 @@
         <v>26</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I14" s="2">
         <v>4</v>
@@ -1721,10 +1716,10 @@
         <v>38</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>29</v>
@@ -1762,13 +1757,13 @@
         <v>26</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I15" s="2">
         <v>4</v>
@@ -1787,10 +1782,10 @@
         <v>38</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q15" s="2" t="s">
         <v>29</v>
@@ -1828,7 +1823,7 @@
         <v>26</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>27</v>
@@ -1856,7 +1851,7 @@
         <v>41</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Q16" s="2" t="s">
         <v>29</v>
@@ -1894,13 +1889,13 @@
         <v>26</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I17" s="2">
         <v>4</v>
@@ -1919,10 +1914,10 @@
         <v>38</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q17" s="2" t="s">
         <v>29</v>
@@ -1960,7 +1955,7 @@
         <v>26</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>27</v>
@@ -1987,10 +1982,10 @@
         <v>38</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>29</v>
@@ -2028,13 +2023,13 @@
         <v>26</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I19" s="2">
         <v>1</v>
@@ -2044,22 +2039,22 @@
       </c>
       <c r="K19" s="2"/>
       <c r="L19" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O19" s="2" t="s">
         <v>41</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="R19" s="2" t="s">
         <v>30</v>
@@ -2091,16 +2086,16 @@
         <v>25</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I20" s="2">
         <v>4</v>
@@ -2122,7 +2117,7 @@
         <v>35</v>
       </c>
       <c r="P20" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="Q20" s="2" t="s">
         <v>29</v>
@@ -2157,16 +2152,16 @@
         <v>25</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>32</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I21" s="2">
         <v>4</v>
@@ -2185,10 +2180,10 @@
         <v>38</v>
       </c>
       <c r="O21" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="P21" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="Q21" s="2" t="s">
         <v>29</v>
@@ -2223,16 +2218,16 @@
         <v>25</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>49</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I22" s="2">
         <v>4</v>
@@ -2254,7 +2249,7 @@
         <v>35</v>
       </c>
       <c r="P22" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="Q22" s="2" t="s">
         <v>29</v>
@@ -2289,16 +2284,16 @@
         <v>25</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>51</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I23" s="2">
         <v>4</v>
@@ -2320,7 +2315,7 @@
         <v>41</v>
       </c>
       <c r="P23" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="Q23" s="2" t="s">
         <v>29</v>
@@ -2348,26 +2343,26 @@
       <c r="B24" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>24</v>
+      <c r="C24" s="3" t="s">
+        <v>96</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="F24" s="2">
-        <v>144</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>95</v>
+        <v>78</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I24" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J24" s="2">
         <v>4</v>
@@ -2379,20 +2374,20 @@
       <c r="M24" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="N24" s="2" t="s">
-        <v>38</v>
+      <c r="N24" s="2">
+        <v>33</v>
       </c>
       <c r="O24" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="P24" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="Q24" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="R24" s="2" t="s">
-        <v>28</v>
+      <c r="R24" s="2">
+        <v>100</v>
       </c>
       <c r="S24" s="2" t="s">
         <v>31</v>
@@ -2401,7 +2396,7 @@
         <v>31</v>
       </c>
       <c r="U24" s="2">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="V24" s="2">
         <v>35</v>

</xml_diff>